<commit_message>
v0.16.32: make the plate say which well each variant sits in
A variant list can state the well of every row, the app issues that file with the wells already written, and the control well is a choice the run honours rather than the preview alone.
</commit_message>
<xml_diff>
--- a/fixtures/mame_demo/KURO_expected.xlsx
+++ b/fixtures/mame_demo/KURO_expected.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fwd List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="expected_mutations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fwd List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="expected_mutations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>M001_I6A_F</t>
+          <t>I6A_F</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>M002_W11C_F</t>
+          <t>W11C_F</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>M003_H16D_F</t>
+          <t>H16D_F</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>M004_V21E_F</t>
+          <t>V21E_F</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>M005_R26F_F</t>
+          <t>R26F_F</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>M006_Q31G_F</t>
+          <t>Q31G_F</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>M007_M36H_F</t>
+          <t>M36H_F</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>M008_N41I_F</t>
+          <t>N41I_F</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>M009_R46K_F</t>
+          <t>R46K_F</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>M010_V51L_F</t>
+          <t>V51L_F</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>M011_H56N_F</t>
+          <t>H56N_F</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>M012_D61P_F</t>
+          <t>D61P_F</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>M013_R66P_F</t>
+          <t>R66P_F</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>M014_H71R_F</t>
+          <t>H71R_F</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>M015_V76R_F</t>
+          <t>V76R_F</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>M016_K81T_F</t>
+          <t>K81T_F</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>M017_I86V_F</t>
+          <t>I86V_F</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>M018_D91W_F</t>
+          <t>D91W_F</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>M019_S96Y_F</t>
+          <t>S96Y_F</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>M020_F101A_F</t>
+          <t>F101A_F</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>M021_W106C_F</t>
+          <t>W106C_F</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>M022_I111D_F</t>
+          <t>I111D_F</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>M023_C116F_F</t>
+          <t>C116F_F</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>M024_Y121F_F</t>
+          <t>Y121F_F</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>M025_R126G_F</t>
+          <t>R126G_F</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>M026_E131I_F</t>
+          <t>E131I_F</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>M027_L136I_F</t>
+          <t>L136I_F</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>M028_K141L_F</t>
+          <t>K141L_F</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>M029_L146M_F</t>
+          <t>L146M_F</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>M030_N151M_F</t>
+          <t>N151M_F</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>M031_Y156N_F</t>
+          <t>Y156N_F</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>M032_N161Q_F</t>
+          <t>N161Q_F</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>M033_W166Q_F</t>
+          <t>W166Q_F</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>M034_V171R_F</t>
+          <t>V171R_F</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>M035_G176T_F</t>
+          <t>G176T_F</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>M036_H181V_F</t>
+          <t>H181V_F</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>M037_N186W_F</t>
+          <t>N186W_F</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>M038_I191Y_F</t>
+          <t>I191Y_F</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>M039_W196A_F</t>
+          <t>W196A_F</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>M040_A201D_F</t>
+          <t>A201D_F</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>M041_C206E_F</t>
+          <t>C206E_F</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>M042_K211E_F</t>
+          <t>K211E_F</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>M043_W216F_F</t>
+          <t>W216F_F</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>M044_Q221G_F</t>
+          <t>Q221G_F</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>M045_N226H_F</t>
+          <t>N226H_F</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>M046_E231K_F</t>
+          <t>E231K_F</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>M047_I236L_F</t>
+          <t>I236L_F</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>M048_F241M_F</t>
+          <t>F241M_F</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>M049_I246N_F</t>
+          <t>I246N_F</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>M050_C251P_F</t>
+          <t>C251P_F</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>M051_G256Q_F</t>
+          <t>G256Q_F</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>M052_P261R_F</t>
+          <t>P261R_F</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>M053_P266S_F</t>
+          <t>P266S_F</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>M054_V271S_F</t>
+          <t>V271S_F</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>M055_H276V_F</t>
+          <t>H276V_F</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>M056_M281W_F</t>
+          <t>M281W_F</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>M057_T286Y_F</t>
+          <t>T286Y_F</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>M058_D291A_F</t>
+          <t>D291A_F</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>M059_I296C_F</t>
+          <t>I296C_F</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>M060_W301D_F</t>
+          <t>W301D_F</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>M061_Q306E_F</t>
+          <t>Q306E_F</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>M062_K311F_F</t>
+          <t>K311F_F</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>M063_P316G_F</t>
+          <t>P316G_F</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>M064_D321I_F</t>
+          <t>D321I_F</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>M065_E326K_F</t>
+          <t>E326K_F</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>M066_K331L_F</t>
+          <t>K331L_F</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>M067_N336L_F</t>
+          <t>N336L_F</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>M068_L341N_F</t>
+          <t>L341N_F</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>M069_L346P_F</t>
+          <t>L346P_F</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>M070_E351Q_F</t>
+          <t>E351Q_F</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>M071_Y356Q_F</t>
+          <t>Y356Q_F</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>M072_T361R_F</t>
+          <t>T361R_F</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>M073_Q366T_F</t>
+          <t>Q366T_F</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>M074_F371V_F</t>
+          <t>F371V_F</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>M075_Q376W_F</t>
+          <t>Q376W_F</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>M076_F381Y_F</t>
+          <t>F381Y_F</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>M077_V386A_F</t>
+          <t>V386A_F</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>M078_L391C_F</t>
+          <t>L391C_F</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>M079_I396D_F</t>
+          <t>I396D_F</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>M080_Y401E_F</t>
+          <t>Y401E_F</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>M081_Q406F_F</t>
+          <t>Q406F_F</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>M082_I411G_F</t>
+          <t>I411G_F</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>M083_C416I_F</t>
+          <t>C416I_F</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>M084_N421I_F</t>
+          <t>N421I_F</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>M085_H426L_F</t>
+          <t>H426L_F</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>M086_K431M_F</t>
+          <t>K431M_F</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>M087_M436N_F</t>
+          <t>M436N_F</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>M088_W441N_F</t>
+          <t>W441N_F</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>M089_Q446P_F</t>
+          <t>Q446P_F</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>M090_T451Q_F</t>
+          <t>T451Q_F</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>M091_K456S_F</t>
+          <t>K456S_F</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>M092_V461S_F</t>
+          <t>V461S_F</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>M093_M466V_F</t>
+          <t>M466V_F</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>M094_T471W_F</t>
+          <t>T471W_F</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>M095_L476Y_F</t>
+          <t>L476Y_F</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4356,47 +4356,6 @@
       <c r="I96" t="inlineStr">
         <is>
           <t>L476Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>H12</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>M096_P481A_F</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>GCGGGCTACTGGCTGCCGGT</t>
-        </is>
-      </c>
-      <c r="D97" t="n">
-        <v>20</v>
-      </c>
-      <c r="E97" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="F97" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>CCG</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>GCG</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>P481A</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4428,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M001_I6A</t>
+          <t>I6A</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4498,7 +4457,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>M001_I6A</t>
+          <t>I6A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4515,7 +4474,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M002_W11C</t>
+          <t>W11C</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4544,7 +4503,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>M002_W11C</t>
+          <t>W11C</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4561,7 +4520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M003_H16D</t>
+          <t>H16D</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4590,7 +4549,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>M003_H16D</t>
+          <t>H16D</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4607,7 +4566,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M004_V21E</t>
+          <t>V21E</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -4636,7 +4595,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>M004_V21E</t>
+          <t>V21E</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -4653,7 +4612,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M005_R26F</t>
+          <t>R26F</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -4682,7 +4641,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>M005_R26F</t>
+          <t>R26F</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4699,7 +4658,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M006_Q31G</t>
+          <t>Q31G</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -4728,7 +4687,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>M006_Q31G</t>
+          <t>Q31G</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4745,7 +4704,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M007_M36H</t>
+          <t>M36H</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4774,7 +4733,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>M007_M36H</t>
+          <t>M36H</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4791,7 +4750,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M008_N41I</t>
+          <t>N41I</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4820,7 +4779,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>M008_N41I</t>
+          <t>N41I</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4837,7 +4796,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M009_R46K</t>
+          <t>R46K</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4866,7 +4825,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>M009_R46K</t>
+          <t>R46K</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4883,7 +4842,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>M010_V51L</t>
+          <t>V51L</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4912,7 +4871,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>M010_V51L</t>
+          <t>V51L</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4929,7 +4888,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>M011_H56N</t>
+          <t>H56N</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4958,7 +4917,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>M011_H56N</t>
+          <t>H56N</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4975,7 +4934,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>M012_D61P</t>
+          <t>D61P</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -5004,7 +4963,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>M012_D61P</t>
+          <t>D61P</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5021,7 +4980,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M013_R66P</t>
+          <t>R66P</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -5050,7 +5009,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>M013_R66P</t>
+          <t>R66P</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5067,7 +5026,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>M014_H71R</t>
+          <t>H71R</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -5096,7 +5055,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>M014_H71R</t>
+          <t>H71R</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5113,7 +5072,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>M015_V76R</t>
+          <t>V76R</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -5142,7 +5101,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>M015_V76R</t>
+          <t>V76R</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5159,7 +5118,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>M016_K81T</t>
+          <t>K81T</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -5188,7 +5147,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>M016_K81T</t>
+          <t>K81T</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5205,7 +5164,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>M017_I86V</t>
+          <t>I86V</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -5234,7 +5193,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>M017_I86V</t>
+          <t>I86V</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5251,7 +5210,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>M018_D91W</t>
+          <t>D91W</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -5280,7 +5239,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>M018_D91W</t>
+          <t>D91W</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5297,7 +5256,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>M019_S96Y</t>
+          <t>S96Y</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -5326,7 +5285,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>M019_S96Y</t>
+          <t>S96Y</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5343,7 +5302,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>M020_F101A</t>
+          <t>F101A</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -5372,7 +5331,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>M020_F101A</t>
+          <t>F101A</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5389,7 +5348,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>M021_W106C</t>
+          <t>W106C</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -5418,7 +5377,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>M021_W106C</t>
+          <t>W106C</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5435,7 +5394,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>M022_I111D</t>
+          <t>I111D</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -5464,7 +5423,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>M022_I111D</t>
+          <t>I111D</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5481,7 +5440,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>M023_C116F</t>
+          <t>C116F</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -5510,7 +5469,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>M023_C116F</t>
+          <t>C116F</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5527,7 +5486,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>M024_Y121F</t>
+          <t>Y121F</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -5556,7 +5515,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>M024_Y121F</t>
+          <t>Y121F</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5573,7 +5532,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>M025_R126G</t>
+          <t>R126G</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -5602,7 +5561,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>M025_R126G</t>
+          <t>R126G</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5619,7 +5578,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>M026_E131I</t>
+          <t>E131I</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -5648,7 +5607,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>M026_E131I</t>
+          <t>E131I</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5665,7 +5624,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>M027_L136I</t>
+          <t>L136I</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -5694,7 +5653,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>M027_L136I</t>
+          <t>L136I</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -5711,7 +5670,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>M028_K141L</t>
+          <t>K141L</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5740,7 +5699,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>M028_K141L</t>
+          <t>K141L</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -5757,7 +5716,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>M029_L146M</t>
+          <t>L146M</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5786,7 +5745,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>M029_L146M</t>
+          <t>L146M</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5803,7 +5762,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>M030_N151M</t>
+          <t>N151M</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -5832,7 +5791,7 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>M030_N151M</t>
+          <t>N151M</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -5849,7 +5808,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>M031_Y156N</t>
+          <t>Y156N</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -5878,7 +5837,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>M031_Y156N</t>
+          <t>Y156N</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -5895,7 +5854,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>M032_N161Q</t>
+          <t>N161Q</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -5924,7 +5883,7 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>M032_N161Q</t>
+          <t>N161Q</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5941,7 +5900,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>M033_W166Q</t>
+          <t>W166Q</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -5970,7 +5929,7 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>M033_W166Q</t>
+          <t>W166Q</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -5987,7 +5946,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>M034_V171R</t>
+          <t>V171R</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -6016,7 +5975,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>M034_V171R</t>
+          <t>V171R</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -6033,7 +5992,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>M035_G176T</t>
+          <t>G176T</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -6062,7 +6021,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>M035_G176T</t>
+          <t>G176T</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -6079,7 +6038,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>M036_H181V</t>
+          <t>H181V</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -6108,7 +6067,7 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>M036_H181V</t>
+          <t>H181V</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -6125,7 +6084,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>M037_N186W</t>
+          <t>N186W</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -6154,7 +6113,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>M037_N186W</t>
+          <t>N186W</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -6171,7 +6130,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>M038_I191Y</t>
+          <t>I191Y</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -6200,7 +6159,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>M038_I191Y</t>
+          <t>I191Y</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -6217,7 +6176,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>M039_W196A</t>
+          <t>W196A</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -6246,7 +6205,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>M039_W196A</t>
+          <t>W196A</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -6263,7 +6222,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>M040_A201D</t>
+          <t>A201D</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -6292,7 +6251,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>M040_A201D</t>
+          <t>A201D</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -6309,7 +6268,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>M041_C206E</t>
+          <t>C206E</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -6338,7 +6297,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>M041_C206E</t>
+          <t>C206E</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -6355,7 +6314,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>M042_K211E</t>
+          <t>K211E</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -6384,7 +6343,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>M042_K211E</t>
+          <t>K211E</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -6401,7 +6360,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>M043_W216F</t>
+          <t>W216F</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -6430,7 +6389,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>M043_W216F</t>
+          <t>W216F</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -6447,7 +6406,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>M044_Q221G</t>
+          <t>Q221G</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -6476,7 +6435,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>M044_Q221G</t>
+          <t>Q221G</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -6493,7 +6452,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>M045_N226H</t>
+          <t>N226H</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -6522,7 +6481,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>M045_N226H</t>
+          <t>N226H</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -6539,7 +6498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>M046_E231K</t>
+          <t>E231K</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -6568,7 +6527,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>M046_E231K</t>
+          <t>E231K</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -6585,7 +6544,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>M047_I236L</t>
+          <t>I236L</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -6614,7 +6573,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>M047_I236L</t>
+          <t>I236L</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -6631,7 +6590,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>M048_F241M</t>
+          <t>F241M</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -6660,7 +6619,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>M048_F241M</t>
+          <t>F241M</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -6677,7 +6636,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>M049_I246N</t>
+          <t>I246N</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -6706,7 +6665,7 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>M049_I246N</t>
+          <t>I246N</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -6723,7 +6682,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>M050_C251P</t>
+          <t>C251P</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -6752,7 +6711,7 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>M050_C251P</t>
+          <t>C251P</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -6769,7 +6728,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>M051_G256Q</t>
+          <t>G256Q</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -6798,7 +6757,7 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>M051_G256Q</t>
+          <t>G256Q</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -6815,7 +6774,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>M052_P261R</t>
+          <t>P261R</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -6844,7 +6803,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>M052_P261R</t>
+          <t>P261R</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -6861,7 +6820,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>M053_P266S</t>
+          <t>P266S</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -6890,7 +6849,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>M053_P266S</t>
+          <t>P266S</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -6907,7 +6866,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>M054_V271S</t>
+          <t>V271S</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -6936,7 +6895,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>M054_V271S</t>
+          <t>V271S</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -6953,7 +6912,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>M055_H276V</t>
+          <t>H276V</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -6982,7 +6941,7 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>M055_H276V</t>
+          <t>H276V</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6999,7 +6958,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>M056_M281W</t>
+          <t>M281W</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -7028,7 +6987,7 @@
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>M056_M281W</t>
+          <t>M281W</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -7045,7 +7004,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>M057_T286Y</t>
+          <t>T286Y</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -7074,7 +7033,7 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>M057_T286Y</t>
+          <t>T286Y</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -7091,7 +7050,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>M058_D291A</t>
+          <t>D291A</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -7120,7 +7079,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>M058_D291A</t>
+          <t>D291A</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -7137,7 +7096,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>M059_I296C</t>
+          <t>I296C</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -7166,7 +7125,7 @@
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>M059_I296C</t>
+          <t>I296C</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -7183,7 +7142,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>M060_W301D</t>
+          <t>W301D</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -7212,7 +7171,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>M060_W301D</t>
+          <t>W301D</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -7229,7 +7188,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>M061_Q306E</t>
+          <t>Q306E</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -7258,7 +7217,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>M061_Q306E</t>
+          <t>Q306E</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7275,7 +7234,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>M062_K311F</t>
+          <t>K311F</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -7304,7 +7263,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>M062_K311F</t>
+          <t>K311F</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7321,7 +7280,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>M063_P316G</t>
+          <t>P316G</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -7350,7 +7309,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>M063_P316G</t>
+          <t>P316G</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7367,7 +7326,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>M064_D321I</t>
+          <t>D321I</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -7396,7 +7355,7 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>M064_D321I</t>
+          <t>D321I</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7413,7 +7372,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>M065_E326K</t>
+          <t>E326K</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -7442,7 +7401,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>M065_E326K</t>
+          <t>E326K</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -7459,7 +7418,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>M066_K331L</t>
+          <t>K331L</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -7488,7 +7447,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>M066_K331L</t>
+          <t>K331L</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -7505,7 +7464,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>M067_N336L</t>
+          <t>N336L</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -7534,7 +7493,7 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>M067_N336L</t>
+          <t>N336L</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7551,7 +7510,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>M068_L341N</t>
+          <t>L341N</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -7580,7 +7539,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>M068_L341N</t>
+          <t>L341N</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7597,7 +7556,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>M069_L346P</t>
+          <t>L346P</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -7626,7 +7585,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>M069_L346P</t>
+          <t>L346P</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7643,7 +7602,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>M070_E351Q</t>
+          <t>E351Q</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -7672,7 +7631,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>M070_E351Q</t>
+          <t>E351Q</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7689,7 +7648,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>M071_Y356Q</t>
+          <t>Y356Q</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -7718,7 +7677,7 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>M071_Y356Q</t>
+          <t>Y356Q</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7735,7 +7694,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>M072_T361R</t>
+          <t>T361R</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -7764,7 +7723,7 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>M072_T361R</t>
+          <t>T361R</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7781,7 +7740,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>M073_Q366T</t>
+          <t>Q366T</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -7810,7 +7769,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>M073_Q366T</t>
+          <t>Q366T</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7827,7 +7786,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>M074_F371V</t>
+          <t>F371V</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -7856,7 +7815,7 @@
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>M074_F371V</t>
+          <t>F371V</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7873,7 +7832,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>M075_Q376W</t>
+          <t>Q376W</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7902,7 +7861,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>M075_Q376W</t>
+          <t>Q376W</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7919,7 +7878,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>M076_F381Y</t>
+          <t>F381Y</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7948,7 +7907,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>M076_F381Y</t>
+          <t>F381Y</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7965,7 +7924,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>M077_V386A</t>
+          <t>V386A</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7994,7 +7953,7 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>M077_V386A</t>
+          <t>V386A</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -8011,7 +7970,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>M078_L391C</t>
+          <t>L391C</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -8040,7 +7999,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>M078_L391C</t>
+          <t>L391C</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8057,7 +8016,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>M079_I396D</t>
+          <t>I396D</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -8086,7 +8045,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>M079_I396D</t>
+          <t>I396D</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -8103,7 +8062,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>M080_Y401E</t>
+          <t>Y401E</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -8132,7 +8091,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>M080_Y401E</t>
+          <t>Y401E</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8149,7 +8108,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>M081_Q406F</t>
+          <t>Q406F</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -8178,7 +8137,7 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>M081_Q406F</t>
+          <t>Q406F</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8195,7 +8154,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>M082_I411G</t>
+          <t>I411G</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -8224,7 +8183,7 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>M082_I411G</t>
+          <t>I411G</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8241,7 +8200,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>M083_C416I</t>
+          <t>C416I</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -8270,7 +8229,7 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>M083_C416I</t>
+          <t>C416I</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8287,7 +8246,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>M084_N421I</t>
+          <t>N421I</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -8316,7 +8275,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>M084_N421I</t>
+          <t>N421I</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8333,7 +8292,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>M085_H426L</t>
+          <t>H426L</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -8362,7 +8321,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>M085_H426L</t>
+          <t>H426L</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8379,7 +8338,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>M086_K431M</t>
+          <t>K431M</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -8408,7 +8367,7 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>M086_K431M</t>
+          <t>K431M</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8425,7 +8384,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>M087_M436N</t>
+          <t>M436N</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -8454,7 +8413,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>M087_M436N</t>
+          <t>M436N</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -8471,7 +8430,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>M088_W441N</t>
+          <t>W441N</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -8500,7 +8459,7 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>M088_W441N</t>
+          <t>W441N</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -8517,7 +8476,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>M089_Q446P</t>
+          <t>Q446P</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -8546,7 +8505,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>M089_Q446P</t>
+          <t>Q446P</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8563,7 +8522,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>M090_T451Q</t>
+          <t>T451Q</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -8592,7 +8551,7 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>M090_T451Q</t>
+          <t>T451Q</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -8609,7 +8568,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>M091_K456S</t>
+          <t>K456S</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -8638,7 +8597,7 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>M091_K456S</t>
+          <t>K456S</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -8655,7 +8614,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>M092_V461S</t>
+          <t>V461S</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -8684,7 +8643,7 @@
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>M092_V461S</t>
+          <t>V461S</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -8701,7 +8660,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>M093_M466V</t>
+          <t>M466V</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -8730,7 +8689,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>M093_M466V</t>
+          <t>M466V</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8747,7 +8706,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>M094_T471W</t>
+          <t>T471W</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -8776,7 +8735,7 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>M094_T471W</t>
+          <t>T471W</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -8793,7 +8752,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>M095_L476Y</t>
+          <t>L476Y</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -8822,7 +8781,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>M095_L476Y</t>
+          <t>L476Y</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -8839,46 +8798,50 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>M096_P481A</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>481</v>
+        <v>0</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>CCG</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>GCG</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>G0</t>
+        </is>
+      </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>M096_P481A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>substitution</t>
+          <t>wt</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>DESIGNED</t>
+          <t>control</t>
         </is>
       </c>
     </row>

</xml_diff>